<commit_message>
Add full daily pipeline with evaluation sync retraining and predictions
</commit_message>
<xml_diff>
--- a/outputs/daily/predictions_2026-06-11.xlsx
+++ b/outputs/daily/predictions_2026-06-11.xlsx
@@ -788,10 +788,10 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>1.916909359667726</v>
+        <v>1.927828074848559</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7393275807356772</v>
+        <v>0.7042589901269826</v>
       </c>
       <c r="M2" t="b">
         <v>1</v>
@@ -815,73 +815,73 @@
         <v>0.7864068322981365</v>
       </c>
       <c r="T2" t="n">
-        <v>0.7318092532806558</v>
+        <v>0.7423105315265203</v>
       </c>
       <c r="U2" t="n">
-        <v>0.1875445745613613</v>
+        <v>0.1826570328702735</v>
       </c>
       <c r="V2" t="n">
-        <v>0.08064617215798289</v>
+        <v>0.07503243560320633</v>
       </c>
       <c r="W2" t="n">
-        <v>0.4836823840600147</v>
+        <v>0.5323487007482608</v>
       </c>
       <c r="X2" t="n">
-        <v>0.376894478795562</v>
+        <v>0.419033168181392</v>
       </c>
       <c r="Y2" t="n">
-        <v>0.6424964446759723</v>
+        <v>0.6539486300909561</v>
       </c>
       <c r="Z2" t="n">
-        <v>0.2309484946387872</v>
+        <v>0.2277122626535442</v>
       </c>
       <c r="AA2" t="n">
-        <v>0.12655506068524</v>
+        <v>0.1183391072554996</v>
       </c>
       <c r="AB2" t="n">
-        <v>0.4955922050970869</v>
+        <v>0.4895925359799504</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.5044077949029131</v>
+        <v>0.5104074640200496</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.4556665485719878</v>
+        <v>0.4417547875153199</v>
       </c>
       <c r="AE2" t="n">
-        <v>0.5443334514280123</v>
+        <v>0.5582452124846802</v>
       </c>
       <c r="AF2" t="n">
-        <v>0.644465</v>
+        <v>0.655855</v>
       </c>
       <c r="AG2" t="n">
-        <v>0.22899</v>
+        <v>0.22585</v>
       </c>
       <c r="AH2" t="n">
-        <v>0.126545</v>
+        <v>0.118295</v>
       </c>
       <c r="AI2" t="n">
-        <v>0.495645</v>
+        <v>0.489275</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0.454655</v>
+        <v>0.440955</v>
       </c>
       <c r="AK2" t="n">
-        <v>1.917905</v>
+        <v>1.928645</v>
       </c>
       <c r="AL2" t="n">
-        <v>0.737865</v>
+        <v>0.70321</v>
       </c>
       <c r="AM2" t="n">
-        <v>2.65577</v>
+        <v>2.631855</v>
       </c>
       <c r="AN2" t="n">
-        <v>0.662765628942001</v>
+        <v>0.6693041226817994</v>
       </c>
       <c r="AO2" t="n">
-        <v>0.2187059329170249</v>
+        <v>0.2161862353288334</v>
       </c>
       <c r="AP2" t="n">
-        <v>0.1185284381409742</v>
+        <v>0.1145096419893673</v>
       </c>
       <c r="AQ2" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="AR2" t="n">
-        <v>0.662765628942001</v>
+        <v>0.6693041226817994</v>
       </c>
       <c r="AS2" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="AT2" t="n">
-        <v>0.1289990622992456</v>
+        <v>0.1336621024289293</v>
       </c>
       <c r="AU2" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="AV2" t="n">
-        <v>0.1246400151703216</v>
+        <v>0.128900320855847</v>
       </c>
       <c r="AW2" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="AX2" t="n">
-        <v>0.1094572579370621</v>
+        <v>0.1074224536443332</v>
       </c>
       <c r="AY2" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="AZ2" t="n">
-        <v>0.09537256464687217</v>
+        <v>0.09413273727484704</v>
       </c>
       <c r="BA2" t="inlineStr">
         <is>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="BB2" t="n">
-        <v>0.08242650330326133</v>
+        <v>0.08589251786859123</v>
       </c>
       <c r="BC2" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="BD2" t="n">
-        <v>0.08016299108623076</v>
+        <v>0.08169429005084833</v>
       </c>
       <c r="BE2" t="inlineStr">
         <is>
@@ -945,23 +945,23 @@
         </is>
       </c>
       <c r="BF2" t="n">
-        <v>0.0609401872757015</v>
+        <v>0.06049057789359785</v>
       </c>
       <c r="BG2" t="inlineStr">
         <is>
+          <t>4-0</t>
+        </is>
+      </c>
+      <c r="BH2" t="n">
+        <v>0.04139650184162543</v>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
           <t>0-1</t>
         </is>
       </c>
-      <c r="BH2" t="n">
-        <v>0.04195925320598854</v>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>4-0</t>
-        </is>
-      </c>
       <c r="BJ2" t="n">
-        <v>0.03950103391667609</v>
+        <v>0.04089069435900088</v>
       </c>
       <c r="BK2" t="inlineStr">
         <is>
@@ -969,7 +969,7 @@
         </is>
       </c>
       <c r="BL2" t="n">
-        <v>0.0367839862293496</v>
+        <v>0.03438783123660032</v>
       </c>
     </row>
     <row r="3">
@@ -1022,10 +1022,10 @@
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>1.517396202607243</v>
+        <v>1.560767614854409</v>
       </c>
       <c r="L3" t="n">
-        <v>1.051122716955019</v>
+        <v>1.065860016684648</v>
       </c>
       <c r="M3" t="b">
         <v>1</v>
@@ -1049,73 +1049,73 @@
         <v>1.133635321100918</v>
       </c>
       <c r="T3" t="n">
-        <v>0.5959237959594534</v>
+        <v>0.6021160820980298</v>
       </c>
       <c r="U3" t="n">
-        <v>0.2555421622836768</v>
+        <v>0.2495490326659355</v>
       </c>
       <c r="V3" t="n">
-        <v>0.1485340417568698</v>
+        <v>0.1483348852360347</v>
       </c>
       <c r="W3" t="n">
-        <v>0.5023151307689514</v>
+        <v>0.5052140846212879</v>
       </c>
       <c r="X3" t="n">
-        <v>0.5179453631976264</v>
+        <v>0.5599628463344619</v>
       </c>
       <c r="Y3" t="n">
-        <v>0.4679755820231893</v>
+        <v>0.4757393596761503</v>
       </c>
       <c r="Z3" t="n">
-        <v>0.2816574923611196</v>
+        <v>0.2770103513311549</v>
       </c>
       <c r="AA3" t="n">
-        <v>0.2503669256156913</v>
+        <v>0.2472502889926944</v>
       </c>
       <c r="AB3" t="n">
-        <v>0.473638545921968</v>
+        <v>0.488233998575669</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.5263614540780319</v>
+        <v>0.511766001424331</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.5200469811965672</v>
+        <v>0.5299466896304029</v>
       </c>
       <c r="AE3" t="n">
-        <v>0.4799530188034328</v>
+        <v>0.4700533103695971</v>
       </c>
       <c r="AF3" t="n">
-        <v>0.467765</v>
+        <v>0.47675</v>
       </c>
       <c r="AG3" t="n">
-        <v>0.280745</v>
+        <v>0.275165</v>
       </c>
       <c r="AH3" t="n">
-        <v>0.25149</v>
+        <v>0.248085</v>
       </c>
       <c r="AI3" t="n">
-        <v>0.472835</v>
+        <v>0.487925</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0.51952</v>
+        <v>0.52871</v>
       </c>
       <c r="AK3" t="n">
-        <v>1.51724</v>
+        <v>1.561345</v>
       </c>
       <c r="AL3" t="n">
-        <v>1.0529</v>
+        <v>1.065945</v>
       </c>
       <c r="AM3" t="n">
-        <v>2.57014</v>
+        <v>2.62729</v>
       </c>
       <c r="AN3" t="n">
-        <v>0.4860525628175918</v>
+        <v>0.4901608073793339</v>
       </c>
       <c r="AO3" t="n">
-        <v>0.2777105505164626</v>
+        <v>0.274451169892762</v>
       </c>
       <c r="AP3" t="n">
-        <v>0.2362368866659456</v>
+        <v>0.2353880227279041</v>
       </c>
       <c r="AQ3" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
         </is>
       </c>
       <c r="AR3" t="n">
-        <v>0.4860525628175918</v>
+        <v>0.4901608073793339</v>
       </c>
       <c r="AS3" t="inlineStr">
         <is>
@@ -1131,7 +1131,7 @@
         </is>
       </c>
       <c r="AT3" t="n">
-        <v>0.134478167292938</v>
+        <v>0.1323431825116791</v>
       </c>
       <c r="AU3" t="inlineStr">
         <is>
@@ -1139,7 +1139,7 @@
         </is>
       </c>
       <c r="AV3" t="n">
-        <v>0.1040816640359461</v>
+        <v>0.1008466487913553</v>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
@@ -1147,23 +1147,23 @@
         </is>
       </c>
       <c r="AX3" t="n">
-        <v>0.09275302744722072</v>
+        <v>0.09388952423227051</v>
       </c>
       <c r="AY3" t="inlineStr">
         <is>
+          <t>2-0</t>
+        </is>
+      </c>
+      <c r="AZ3" t="n">
+        <v>0.08808804417329902</v>
+      </c>
+      <c r="BA3" t="inlineStr">
+        <is>
           <t>0-0</t>
         </is>
       </c>
-      <c r="AZ3" t="n">
-        <v>0.08887432117557359</v>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>2-0</t>
-        </is>
-      </c>
       <c r="BB3" t="n">
-        <v>0.0882418636293158</v>
+        <v>0.08435320594491134</v>
       </c>
       <c r="BC3" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="BD3" t="n">
-        <v>0.06834225213532714</v>
+        <v>0.06505393774751252</v>
       </c>
       <c r="BE3" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="BF3" t="n">
-        <v>0.06425138935276568</v>
+        <v>0.06411786669090805</v>
       </c>
       <c r="BG3" t="inlineStr">
         <is>
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="BH3" t="n">
-        <v>0.04874740710806305</v>
+        <v>0.05003654493236076</v>
       </c>
       <c r="BI3" t="inlineStr">
         <is>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
       <c r="BJ3" t="n">
-        <v>0.04691436387624606</v>
+        <v>0.04884657626527205</v>
       </c>
       <c r="BK3" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         </is>
       </c>
       <c r="BL3" t="n">
-        <v>0.04463262292737001</v>
+        <v>0.0458283222005166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add Telegram notifications and daily script integration
</commit_message>
<xml_diff>
--- a/outputs/daily/predictions_2026-06-11.xlsx
+++ b/outputs/daily/predictions_2026-06-11.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BL3"/>
+  <dimension ref="A1:BW2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -639,100 +639,155 @@
       </c>
       <c r="AS1" t="inlineStr">
         <is>
+          <t>has_value_data</t>
+        </is>
+      </c>
+      <c r="AT1" t="inlineStr">
+        <is>
+          <t>best_value_market</t>
+        </is>
+      </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>best_value_odds</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>best_value_probability</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>best_value_edge</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>best_value_ev</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>best_edge_market</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>best_edge_odds</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>best_edge_probability</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>best_edge</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>best_edge_ev</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
           <t>top_score_1</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="BE1" t="inlineStr">
         <is>
           <t>top_score_1_prob</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="BF1" t="inlineStr">
         <is>
           <t>top_score_2</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="BG1" t="inlineStr">
         <is>
           <t>top_score_2_prob</t>
         </is>
       </c>
-      <c r="AW1" t="inlineStr">
+      <c r="BH1" t="inlineStr">
         <is>
           <t>top_score_3</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="BI1" t="inlineStr">
         <is>
           <t>top_score_3_prob</t>
         </is>
       </c>
-      <c r="AY1" t="inlineStr">
+      <c r="BJ1" t="inlineStr">
         <is>
           <t>top_score_4</t>
         </is>
       </c>
-      <c r="AZ1" t="inlineStr">
+      <c r="BK1" t="inlineStr">
         <is>
           <t>top_score_4_prob</t>
         </is>
       </c>
-      <c r="BA1" t="inlineStr">
+      <c r="BL1" t="inlineStr">
         <is>
           <t>top_score_5</t>
         </is>
       </c>
-      <c r="BB1" t="inlineStr">
+      <c r="BM1" t="inlineStr">
         <is>
           <t>top_score_5_prob</t>
         </is>
       </c>
-      <c r="BC1" t="inlineStr">
+      <c r="BN1" t="inlineStr">
         <is>
           <t>top_score_6</t>
         </is>
       </c>
-      <c r="BD1" t="inlineStr">
+      <c r="BO1" t="inlineStr">
         <is>
           <t>top_score_6_prob</t>
         </is>
       </c>
-      <c r="BE1" t="inlineStr">
+      <c r="BP1" t="inlineStr">
         <is>
           <t>top_score_7</t>
         </is>
       </c>
-      <c r="BF1" t="inlineStr">
+      <c r="BQ1" t="inlineStr">
         <is>
           <t>top_score_7_prob</t>
         </is>
       </c>
-      <c r="BG1" t="inlineStr">
+      <c r="BR1" t="inlineStr">
         <is>
           <t>top_score_8</t>
         </is>
       </c>
-      <c r="BH1" t="inlineStr">
+      <c r="BS1" t="inlineStr">
         <is>
           <t>top_score_8_prob</t>
         </is>
       </c>
-      <c r="BI1" t="inlineStr">
+      <c r="BT1" t="inlineStr">
         <is>
           <t>top_score_9</t>
         </is>
       </c>
-      <c r="BJ1" t="inlineStr">
+      <c r="BU1" t="inlineStr">
         <is>
           <t>top_score_9_prob</t>
         </is>
       </c>
-      <c r="BK1" t="inlineStr">
+      <c r="BV1" t="inlineStr">
         <is>
           <t>top_score_10</t>
         </is>
       </c>
-      <c r="BL1" t="inlineStr">
+      <c r="BW1" t="inlineStr">
         <is>
           <t>top_score_10_prob</t>
         </is>
@@ -891,319 +946,122 @@
       <c r="AR2" t="n">
         <v>0.6693041226817994</v>
       </c>
-      <c r="AS2" t="inlineStr">
+      <c r="AS2" t="b">
+        <v>1</v>
+      </c>
+      <c r="AT2" t="inlineStr">
+        <is>
+          <t>HOME</t>
+        </is>
+      </c>
+      <c r="AU2" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="AV2" t="n">
+        <v>0.6693041226817994</v>
+      </c>
+      <c r="AW2" t="n">
+        <v>0.02414283235921877</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>0.03742139015678903</v>
+      </c>
+      <c r="AY2" t="inlineStr">
+        <is>
+          <t>HOME</t>
+        </is>
+      </c>
+      <c r="AZ2" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0.6693041226817994</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0.02414283235921877</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0.03742139015678903</v>
+      </c>
+      <c r="BD2" t="inlineStr">
         <is>
           <t>2-0</t>
         </is>
       </c>
-      <c r="AT2" t="n">
+      <c r="BE2" t="n">
         <v>0.1336621024289293</v>
       </c>
-      <c r="AU2" t="inlineStr">
+      <c r="BF2" t="inlineStr">
         <is>
           <t>1-0</t>
         </is>
       </c>
-      <c r="AV2" t="n">
+      <c r="BG2" t="n">
         <v>0.128900320855847</v>
       </c>
-      <c r="AW2" t="inlineStr">
+      <c r="BH2" t="inlineStr">
         <is>
           <t>1-1</t>
         </is>
       </c>
-      <c r="AX2" t="n">
+      <c r="BI2" t="n">
         <v>0.1074224536443332</v>
       </c>
-      <c r="AY2" t="inlineStr">
+      <c r="BJ2" t="inlineStr">
         <is>
           <t>2-1</t>
         </is>
       </c>
-      <c r="AZ2" t="n">
+      <c r="BK2" t="n">
         <v>0.09413273727484704</v>
       </c>
-      <c r="BA2" t="inlineStr">
+      <c r="BL2" t="inlineStr">
         <is>
           <t>3-0</t>
         </is>
       </c>
-      <c r="BB2" t="n">
+      <c r="BM2" t="n">
         <v>0.08589251786859123</v>
       </c>
-      <c r="BC2" t="inlineStr">
+      <c r="BN2" t="inlineStr">
         <is>
           <t>0-0</t>
         </is>
       </c>
-      <c r="BD2" t="n">
+      <c r="BO2" t="n">
         <v>0.08169429005084833</v>
       </c>
-      <c r="BE2" t="inlineStr">
+      <c r="BP2" t="inlineStr">
         <is>
           <t>3-1</t>
         </is>
       </c>
-      <c r="BF2" t="n">
+      <c r="BQ2" t="n">
         <v>0.06049057789359785</v>
       </c>
-      <c r="BG2" t="inlineStr">
+      <c r="BR2" t="inlineStr">
         <is>
           <t>4-0</t>
         </is>
       </c>
-      <c r="BH2" t="n">
+      <c r="BS2" t="n">
         <v>0.04139650184162543</v>
       </c>
-      <c r="BI2" t="inlineStr">
+      <c r="BT2" t="inlineStr">
         <is>
           <t>0-1</t>
         </is>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BU2" t="n">
         <v>0.04089069435900088</v>
       </c>
-      <c r="BK2" t="inlineStr">
+      <c r="BV2" t="inlineStr">
         <is>
           <t>1-2</t>
         </is>
       </c>
-      <c r="BL2" t="n">
+      <c r="BW2" t="n">
         <v>0.03438783123660032</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>WC2026-002</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-06-11T22:00:00+00:00</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Group Stage</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Estadio Akron</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Guadalajara</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Czechia</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="n">
-        <v>1.560767614854409</v>
-      </c>
-      <c r="L3" t="n">
-        <v>1.065860016684648</v>
-      </c>
-      <c r="M3" t="b">
-        <v>1</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.4012133468149647</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.2946410515672397</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.3041456016177958</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.4545454545454546</v>
-      </c>
-      <c r="R3" t="n">
-        <v>1.356364678899083</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1.133635321100918</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.6021160820980298</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.2495490326659355</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0.1483348852360347</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.5052140846212879</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0.5599628463344619</v>
-      </c>
-      <c r="Y3" t="n">
-        <v>0.4757393596761503</v>
-      </c>
-      <c r="Z3" t="n">
-        <v>0.2770103513311549</v>
-      </c>
-      <c r="AA3" t="n">
-        <v>0.2472502889926944</v>
-      </c>
-      <c r="AB3" t="n">
-        <v>0.488233998575669</v>
-      </c>
-      <c r="AC3" t="n">
-        <v>0.511766001424331</v>
-      </c>
-      <c r="AD3" t="n">
-        <v>0.5299466896304029</v>
-      </c>
-      <c r="AE3" t="n">
-        <v>0.4700533103695971</v>
-      </c>
-      <c r="AF3" t="n">
-        <v>0.47675</v>
-      </c>
-      <c r="AG3" t="n">
-        <v>0.275165</v>
-      </c>
-      <c r="AH3" t="n">
-        <v>0.248085</v>
-      </c>
-      <c r="AI3" t="n">
-        <v>0.487925</v>
-      </c>
-      <c r="AJ3" t="n">
-        <v>0.52871</v>
-      </c>
-      <c r="AK3" t="n">
-        <v>1.561345</v>
-      </c>
-      <c r="AL3" t="n">
-        <v>1.065945</v>
-      </c>
-      <c r="AM3" t="n">
-        <v>2.62729</v>
-      </c>
-      <c r="AN3" t="n">
-        <v>0.4901608073793339</v>
-      </c>
-      <c r="AO3" t="n">
-        <v>0.274451169892762</v>
-      </c>
-      <c r="AP3" t="n">
-        <v>0.2353880227279041</v>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>HOME</t>
-        </is>
-      </c>
-      <c r="AR3" t="n">
-        <v>0.4901608073793339</v>
-      </c>
-      <c r="AS3" t="inlineStr">
-        <is>
-          <t>1-1</t>
-        </is>
-      </c>
-      <c r="AT3" t="n">
-        <v>0.1323431825116791</v>
-      </c>
-      <c r="AU3" t="inlineStr">
-        <is>
-          <t>1-0</t>
-        </is>
-      </c>
-      <c r="AV3" t="n">
-        <v>0.1008466487913553</v>
-      </c>
-      <c r="AW3" t="inlineStr">
-        <is>
-          <t>2-1</t>
-        </is>
-      </c>
-      <c r="AX3" t="n">
-        <v>0.09388952423227051</v>
-      </c>
-      <c r="AY3" t="inlineStr">
-        <is>
-          <t>2-0</t>
-        </is>
-      </c>
-      <c r="AZ3" t="n">
-        <v>0.08808804417329902</v>
-      </c>
-      <c r="BA3" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
-      <c r="BB3" t="n">
-        <v>0.08435320594491134</v>
-      </c>
-      <c r="BC3" t="inlineStr">
-        <is>
-          <t>0-1</t>
-        </is>
-      </c>
-      <c r="BD3" t="n">
-        <v>0.06505393774751252</v>
-      </c>
-      <c r="BE3" t="inlineStr">
-        <is>
-          <t>1-2</t>
-        </is>
-      </c>
-      <c r="BF3" t="n">
-        <v>0.06411786669090805</v>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>2-2</t>
-        </is>
-      </c>
-      <c r="BH3" t="n">
-        <v>0.05003654493236076</v>
-      </c>
-      <c r="BI3" t="inlineStr">
-        <is>
-          <t>3-1</t>
-        </is>
-      </c>
-      <c r="BJ3" t="n">
-        <v>0.04884657626527205</v>
-      </c>
-      <c r="BK3" t="inlineStr">
-        <is>
-          <t>3-0</t>
-        </is>
-      </c>
-      <c r="BL3" t="n">
-        <v>0.0458283222005166</v>
       </c>
     </row>
   </sheetData>

</xml_diff>